<commit_message>
feat: Add IDEX printhead designs, image analysis scripts, and related documentation/assets.
</commit_message>
<xml_diff>
--- a/Documentation/Experiments/Bi-directional Specimen Testing.xlsx
+++ b/Documentation/Experiments/Bi-directional Specimen Testing.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
   <si>
     <t xml:space="preserve">Print Speed</t>
   </si>
@@ -32,6 +32,18 @@
   </si>
   <si>
     <t xml:space="preserve">Tensile Strength / N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longitudinal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vertical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150mm</t>
   </si>
   <si>
     <t xml:space="preserve">Layer deposition interval / s   at distance x mm</t>
@@ -225,7 +237,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -271,7 +283,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -316,10 +336,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -505,7 +521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
@@ -613,240 +629,323 @@
       <c r="B4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="12" t="n">
-        <v>245</v>
-      </c>
-      <c r="D4" s="13" t="n">
-        <v>241.5</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>259.5</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>254.5</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>253</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>287</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>258</v>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>270.5</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>252.5</v>
-      </c>
-      <c r="L4" s="13" t="n">
-        <v>263.5</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>220</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>225</v>
-      </c>
-      <c r="P4" s="5"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="11"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="17"/>
-      <c r="P5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="23.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="P5" s="13"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="14" t="n">
+        <v>245</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>241.5</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>259.5</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>254.5</v>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>253</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>287</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>258</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>270.5</v>
+      </c>
+      <c r="K6" s="14" t="n">
+        <v>252.5</v>
+      </c>
+      <c r="L6" s="15" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="M6" s="14" t="n">
+        <v>220</v>
+      </c>
+      <c r="N6" s="16" t="n">
+        <v>225</v>
+      </c>
+      <c r="O6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="P6" s="13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="17" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>105</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>125</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="H7" s="18" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>120</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="L7" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="M7" s="17" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="N7" s="19" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="O7" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="P7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O9" s="0"/>
+      <c r="P9" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="23.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="21" t="n">
         <v>150</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="21" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="C17" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="21" t="n">
         <v>150</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C20" s="12" t="n">
         <f aca="false">75/C2</f>
         <v>15</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D20" s="12" t="n">
         <f aca="false">75/D2</f>
         <v>7.5</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E20" s="12" t="n">
         <f aca="false">75/E2</f>
         <v>5</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F20" s="12" t="n">
         <f aca="false">75/F2</f>
         <v>3.75</v>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G20" s="12" t="n">
         <f aca="false">75/G2</f>
         <v>3</v>
       </c>
-      <c r="H12" s="23" t="n">
+      <c r="H20" s="12" t="n">
         <f aca="false">75/H2</f>
         <v>2.5</v>
       </c>
-      <c r="I12" s="23" t="n">
+      <c r="I20" s="12" t="n">
         <f aca="false">75/I2</f>
         <v>2.14285714285714</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J20" s="12" t="n">
         <f aca="false">75/J2</f>
         <v>1.875</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="K20" s="12" t="n">
         <f aca="false">75/K2</f>
         <v>1.66666666666667</v>
       </c>
-      <c r="L12" s="23" t="n">
+      <c r="L20" s="12" t="n">
         <f aca="false">75/L2</f>
         <v>1.5</v>
       </c>
-      <c r="M12" s="23" t="n">
+      <c r="M20" s="12" t="n">
         <f aca="false">75/M2</f>
         <v>1.36363636363636</v>
       </c>
-      <c r="N12" s="23" t="n">
+      <c r="N20" s="12" t="n">
         <f aca="false">75/N2</f>
         <v>1.25</v>
       </c>
-      <c r="O12" s="18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+      <c r="O20" s="20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
+  <mergeCells count="5">
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>